<commit_message>
Actualización Back Productos Financiados 01-may-2026
</commit_message>
<xml_diff>
--- a/Productos Financiados/Documentos/Relación de horas.xlsx
+++ b/Productos Financiados/Documentos/Relación de horas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Terceros\SisArrendaCredito\Productos Financiados\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD78FF37-AEA4-42B0-8FEC-C6EE075FA599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E36E848-4D67-4A95-B356-070BCB40255F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7A6E54A7-1C89-4907-9763-05848EEF796F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Fecha</t>
   </si>
@@ -76,6 +76,20 @@
 3.	Creación de Script de Alta de Catalogo Mensajes Errores
 4.	Creación Procedimiento spa_SO_RelUnidadProductoFinTbl
 5.	Pruebas del Procedimiento spa_SO_RelUnidadProductoFinTbl</t>
+  </si>
+  <si>
+    <t>1. Creación Objeto spu_SO_RelUnidadProductoFinTbl
+2. Creación Objeto spc_SO_RelUnidadProductoFinTbl
+3. Creación Objeto spd_SO_RelUnidadProductoFinTbl
+4. Creación Objeto TrinsSO_RelUnidadProductoFinTbl
+5. Creación Objeto SO_RelUnidadProductoFinDetTbl
+6. Creación Objeto spa_SO_RelUnidadProductoFinDetDetTbl
+7. Pruebas de los objetos generados</t>
+  </si>
+  <si>
+    <t>1. Creación Objeto spu_SO_RelUnidadProductoFinDetTbl
+2. Creación Objeto spc_SO_RelUnidadProductoFinDetTbl
+3. Creación Objeto spd_SO_RelUnidadProductoFinDetTbl</t>
   </si>
 </sst>
 </file>
@@ -138,17 +152,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -268,8 +282,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}" name="Tabla1" displayName="Tabla1" ref="A9:F14" totalsRowCount="1" headerRowDxfId="10">
-  <autoFilter ref="A9:F13" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}" name="Tabla1" displayName="Tabla1" ref="A9:F18" totalsRowCount="1" headerRowDxfId="10">
+  <autoFilter ref="A9:F17" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{34329E0F-16A5-4583-9308-70D1D98D832B}" name="Fecha" dataDxfId="9" totalsRowDxfId="5"/>
     <tableColumn id="2" xr3:uid="{AD703B33-1671-4278-8CD6-BE420E9DC524}" name="Descripción" dataDxfId="8" totalsRowDxfId="4"/>
@@ -599,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E6A9BD7-1DE2-458E-BBC1-4A16120DB6D2}">
-  <dimension ref="A7:F14"/>
+  <dimension ref="A7:F18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="65" customWidth="1"/>
@@ -608,14 +622,14 @@
   </cols>
   <sheetData>
     <row r="7" spans="1:6" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -647,10 +661,10 @@
       <c r="C10" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="7">
         <v>0.70833333333333337</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="7">
         <v>0.75</v>
       </c>
       <c r="F10" s="5">
@@ -667,10 +681,10 @@
       <c r="C11" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="9">
+      <c r="D11" s="8">
         <v>0.66666666666666663</v>
       </c>
-      <c r="E11" s="9">
+      <c r="E11" s="8">
         <v>0.70833333333333304</v>
       </c>
       <c r="F11" s="5">
@@ -687,10 +701,10 @@
       <c r="C12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D12" s="8">
+      <c r="D12" s="7">
         <v>0.54166666666666663</v>
       </c>
-      <c r="E12" s="8">
+      <c r="E12" s="7">
         <v>0.58333333333333337</v>
       </c>
       <c r="F12" s="5">
@@ -699,29 +713,79 @@
     </row>
     <row r="13" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>11</v>
       </c>
       <c r="C13" s="4"/>
-      <c r="D13" s="9">
+      <c r="D13" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="8">
         <v>0.83333333333333337</v>
       </c>
       <c r="F13" s="5">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="5"/>
-      <c r="B14" s="3"/>
+    <row r="14" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>46143</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>12</v>
+      </c>
       <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
+      <c r="D14" s="8">
+        <v>0.36805555555555558</v>
+      </c>
+      <c r="E14" s="8">
+        <v>0.63888888888888884</v>
+      </c>
       <c r="F14" s="5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+      <c r="B16" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" s="4"/>
+      <c r="D16" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="E16" s="8">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F16" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="5"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="5">
         <f>SUBTOTAL(109,Tabla1[Horas])</f>
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización Back Productos Financiados 4-may-2026
</commit_message>
<xml_diff>
--- a/Productos Financiados/Documentos/Relación de horas.xlsx
+++ b/Productos Financiados/Documentos/Relación de horas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Terceros\SisArrendaCredito\Productos Financiados\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E36E848-4D67-4A95-B356-070BCB40255F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05792BC-B503-42C0-8360-247A8EC2EF59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7A6E54A7-1C89-4907-9763-05848EEF796F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>Fecha</t>
   </si>
@@ -87,9 +87,23 @@
 7. Pruebas de los objetos generados</t>
   </si>
   <si>
-    <t>1. Creación Objeto spu_SO_RelUnidadProductoFinDetTbl
+    <t xml:space="preserve">1. Creación Objeto spu_SO_RelUnidadProductoFinDetTbl
 2. Creación Objeto spc_SO_RelUnidadProductoFinDetTbl
-3. Creación Objeto spd_SO_RelUnidadProductoFinDetTbl</t>
+</t>
+  </si>
+  <si>
+    <t>1. Creación Objeto spd_SO_RelUnidadProductoFinDetTbl
+2.  TrinsSO_RelUnidadProductoFinDetTbl.sql</t>
+  </si>
+  <si>
+    <t>1.- Creación Objeto SO_RelUnidadProductoFinAmorTbl
+2.- Creación Objeto spa_SO_RelUnidadProductoFinAmorTbl
+3.- Creación Objeto spc_SO_RelUnidadProductoFinAmorTbl
+4.- Creación Objeto spd_SO_RelUnidadProductoFinAmorTbl
+5.- Creación Objeto TrinsSO_RelUnidadProductoFinAmorTbl
+6.- Ajuste al Script del Catalogo de Errores.
+7.- Generación Diagrama Entidad-Relación.
+8.- Junta de Revisión con Miguel Zamora"</t>
   </si>
 </sst>
 </file>
@@ -711,7 +725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="87" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="9" t="s">
         <v>11</v>
@@ -727,7 +741,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>46143</v>
       </c>
@@ -745,37 +759,57 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="3"/>
+      <c r="B15" s="3" t="s">
+        <v>13</v>
+      </c>
       <c r="C15" s="4"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
+      <c r="D15" s="8">
+        <v>0.75</v>
+      </c>
+      <c r="E15" s="8">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F15" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>46143</v>
+      </c>
       <c r="B16" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="8">
-        <v>0.75</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="E16" s="8">
-        <v>0.79166666666666663</v>
+        <v>0.46875</v>
       </c>
       <c r="F16" s="5">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="3"/>
+    <row r="17" spans="1:6" ht="129.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>46146</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>15</v>
+      </c>
       <c r="C17" s="4"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="5"/>
+      <c r="D17" s="8">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="E17" s="8">
+        <v>0.64236111111111116</v>
+      </c>
+      <c r="F17" s="5">
+        <v>4</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
@@ -785,7 +819,7 @@
       <c r="E18" s="4"/>
       <c r="F18" s="5">
         <f>SUBTOTAL(109,Tabla1[Horas])</f>
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización Back Productos Financiados 05-may-2026
</commit_message>
<xml_diff>
--- a/Productos Financiados/Documentos/Relación de horas.xlsx
+++ b/Productos Financiados/Documentos/Relación de horas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Terceros\SisArrendaCredito\Productos Financiados\Documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D05792BC-B503-42C0-8360-247A8EC2EF59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EA66711-732D-4C7E-8633-7D853BCF0503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7A6E54A7-1C89-4907-9763-05848EEF796F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
     <t>Fecha</t>
   </si>
@@ -104,6 +104,9 @@
 6.- Ajuste al Script del Catalogo de Errores.
 7.- Generación Diagrama Entidad-Relación.
 8.- Junta de Revisión con Miguel Zamora"</t>
+  </si>
+  <si>
+    <t>Generación de documentación del proceso de financiación de productos relacionaos a una unidad</t>
   </si>
 </sst>
 </file>
@@ -296,8 +299,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}" name="Tabla1" displayName="Tabla1" ref="A9:F18" totalsRowCount="1" headerRowDxfId="10">
-  <autoFilter ref="A9:F17" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}" name="Tabla1" displayName="Tabla1" ref="A9:F19" totalsRowCount="1" headerRowDxfId="10">
+  <autoFilter ref="A9:F18" xr:uid="{63582B99-8CCA-4D66-89D7-648F8ECCB686}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{34329E0F-16A5-4583-9308-70D1D98D832B}" name="Fecha" dataDxfId="9" totalsRowDxfId="5"/>
     <tableColumn id="2" xr3:uid="{AD703B33-1671-4278-8CD6-BE420E9DC524}" name="Descripción" dataDxfId="8" totalsRowDxfId="4"/>
@@ -627,7 +630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E6A9BD7-1DE2-458E-BBC1-4A16120DB6D2}">
-  <dimension ref="A7:F18"/>
+  <dimension ref="A7:F19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="65" customWidth="1"/>
@@ -811,15 +814,33 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="5"/>
-      <c r="B18" s="3"/>
+    <row r="18" spans="1:6" ht="129.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>46147</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
+      <c r="D18" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="E18" s="8">
+        <v>0.58333333333333337</v>
+      </c>
       <c r="F18" s="5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="5"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="5">
         <f>SUBTOTAL(109,Tabla1[Horas])</f>
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>